<commit_message>
feat: AI auto-pilot recorder — auto_recorder.ts reads JSON steps, performs all actions in browser, writes verified spec files; fix Built-ins typo in logic_containers_testcases.json
</commit_message>
<xml_diff>
--- a/manualtestcasedoc/LogicContainers.xlsx
+++ b/manualtestcasedoc/LogicContainers.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
   <si>
     <t>S.No</t>
   </si>
@@ -141,10 +141,10 @@
     <t>Step10</t>
   </si>
   <si>
-    <t>Click Build-ins Subtab</t>
+    <t>Click "Built-ins" Subtab</t>
   </si>
   <si>
-    <t>Build-ins subtab should be clicked</t>
+    <t>Built-ins subtab should be clicked</t>
   </si>
   <si>
     <t>Step11</t>
@@ -286,6 +286,9 @@
   </si>
   <si>
     <t>Validate the set variable container is working</t>
+  </si>
+  <si>
+    <t>"Built-ins" subtab should be clicked</t>
   </si>
   <si>
     <t>Drag "Set Variable" into Trigger box</t>
@@ -2116,7 +2119,7 @@
         <v>42</v>
       </c>
       <c r="G38" s="13" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="H38" s="8"/>
       <c r="I38" s="10"/>
@@ -2183,10 +2186,10 @@
         <v>47</v>
       </c>
       <c r="F40" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G40" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H40" s="8"/>
       <c r="I40" s="10"/>
@@ -2218,10 +2221,10 @@
         <v>50</v>
       </c>
       <c r="F41" s="8" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H41" s="8"/>
       <c r="I41" s="10"/>
@@ -2288,10 +2291,10 @@
         <v>56</v>
       </c>
       <c r="F43" s="15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G43" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H43" s="8"/>
       <c r="I43" s="10"/>
@@ -2323,10 +2326,10 @@
         <v>59</v>
       </c>
       <c r="F44" s="15" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G44" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H44" s="8"/>
       <c r="I44" s="10"/>
@@ -2358,10 +2361,10 @@
         <v>62</v>
       </c>
       <c r="F45" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G45" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H45" s="8"/>
       <c r="I45" s="10"/>
@@ -2393,10 +2396,10 @@
         <v>65</v>
       </c>
       <c r="F46" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G46" s="16" t="s">
         <v>101</v>
-      </c>
-      <c r="G46" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="H46" s="8"/>
       <c r="I46" s="10"/>
@@ -2463,10 +2466,10 @@
         <v>71</v>
       </c>
       <c r="F48" s="15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G48" s="16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H48" s="8"/>
       <c r="I48" s="10"/>
@@ -2498,10 +2501,10 @@
         <v>74</v>
       </c>
       <c r="F49" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H49" s="8"/>
       <c r="I49" s="10"/>
@@ -2533,10 +2536,10 @@
         <v>77</v>
       </c>
       <c r="F50" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G50" s="9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H50" s="8"/>
       <c r="I50" s="10"/>
@@ -2568,10 +2571,10 @@
         <v>80</v>
       </c>
       <c r="F51" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H51" s="8"/>
       <c r="I51" s="10"/>
@@ -2603,10 +2606,10 @@
         <v>83</v>
       </c>
       <c r="F52" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G52" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H52" s="8"/>
       <c r="I52" s="10"/>
@@ -2638,10 +2641,10 @@
         <v>86</v>
       </c>
       <c r="F53" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G53" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H53" s="8"/>
       <c r="I53" s="10"/>
@@ -2670,13 +2673,13 @@
         <v>13</v>
       </c>
       <c r="E54" s="12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F54" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G54" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H54" s="8"/>
       <c r="I54" s="10"/>
@@ -2705,13 +2708,13 @@
         <v>13</v>
       </c>
       <c r="E55" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F55" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H55" s="8"/>
       <c r="I55" s="10"/>
@@ -2737,10 +2740,10 @@
         <v>3.0</v>
       </c>
       <c r="B56" s="8" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="C56" s="8" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="D56" s="8" t="s">
         <v>11</v>
@@ -3341,7 +3344,7 @@
         <v>42</v>
       </c>
       <c r="G66" s="13" t="s">
-        <v>43</v>
+        <v>91</v>
       </c>
       <c r="H66" s="8"/>
       <c r="I66" s="10"/>
@@ -3462,10 +3465,10 @@
         <v>47</v>
       </c>
       <c r="F68" s="8" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="G68" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="H68" s="8"/>
       <c r="I68" s="10"/>
@@ -3524,10 +3527,10 @@
         <v>50</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="G69" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H69" s="8"/>
       <c r="I69" s="10"/>
@@ -3648,10 +3651,10 @@
         <v>56</v>
       </c>
       <c r="F71" s="15" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="H71" s="8"/>
       <c r="I71" s="10"/>
@@ -3710,10 +3713,10 @@
         <v>59</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="G72" s="16" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="H72" s="8"/>
       <c r="I72" s="10"/>
@@ -3772,10 +3775,10 @@
         <v>62</v>
       </c>
       <c r="F73" s="15" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="H73" s="8"/>
       <c r="I73" s="10"/>
@@ -3834,10 +3837,10 @@
         <v>65</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="G74" s="16" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="H74" s="8"/>
       <c r="I74" s="10"/>
@@ -3896,10 +3899,10 @@
         <v>68</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="H75" s="8"/>
       <c r="I75" s="10"/>
@@ -3958,10 +3961,10 @@
         <v>71</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="G76" s="16" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="H76" s="8"/>
       <c r="I76" s="10"/>
@@ -4082,10 +4085,10 @@
         <v>77</v>
       </c>
       <c r="F78" s="15" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="G78" s="16" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="H78" s="8"/>
       <c r="I78" s="10"/>
@@ -4144,10 +4147,10 @@
         <v>80</v>
       </c>
       <c r="F79" s="15" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="G79" s="16" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="H79" s="8"/>
       <c r="I79" s="10"/>
@@ -4206,10 +4209,10 @@
         <v>83</v>
       </c>
       <c r="F80" s="17" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G80" s="16" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="H80" s="8"/>
       <c r="I80" s="10"/>
@@ -4268,10 +4271,10 @@
         <v>86</v>
       </c>
       <c r="F81" s="15" t="s">
+        <v>102</v>
+      </c>
+      <c r="G81" s="16" t="s">
         <v>101</v>
-      </c>
-      <c r="G81" s="16" t="s">
-        <v>100</v>
       </c>
       <c r="H81" s="8"/>
       <c r="I81" s="10"/>
@@ -4327,7 +4330,7 @@
         <v>13</v>
       </c>
       <c r="E82" s="12" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F82" s="15" t="s">
         <v>39</v>
@@ -4389,13 +4392,13 @@
         <v>13</v>
       </c>
       <c r="E83" s="12" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="F83" s="15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="G83" s="16" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="H83" s="8"/>
       <c r="I83" s="10"/>
@@ -4451,13 +4454,13 @@
         <v>13</v>
       </c>
       <c r="E84" s="12" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="F84" s="8" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="G84" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="H84" s="8"/>
       <c r="I84" s="10"/>
@@ -4513,13 +4516,13 @@
         <v>13</v>
       </c>
       <c r="E85" s="12" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F85" s="8" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="G85" s="9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="H85" s="8"/>
       <c r="I85" s="10"/>
@@ -4575,13 +4578,13 @@
         <v>13</v>
       </c>
       <c r="E86" s="12" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="F86" s="8" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="G86" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="H86" s="8"/>
       <c r="I86" s="10"/>
@@ -4637,13 +4640,13 @@
         <v>13</v>
       </c>
       <c r="E87" s="12" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="F87" s="8" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="G87" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="H87" s="8"/>
       <c r="I87" s="10"/>
@@ -4699,13 +4702,13 @@
         <v>13</v>
       </c>
       <c r="E88" s="12" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F88" s="8" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="G88" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="H88" s="8"/>
       <c r="I88" s="10"/>
@@ -4761,13 +4764,13 @@
         <v>13</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="F89" s="8" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G89" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="H89" s="8"/>
       <c r="I89" s="10"/>
@@ -4823,13 +4826,13 @@
         <v>13</v>
       </c>
       <c r="E90" s="12" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="F90" s="8" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="G90" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="H90" s="8"/>
       <c r="I90" s="10"/>

</xml_diff>

<commit_message>
feat: add TC4 Delay Container, fix TC2/TC3/TC5 selectors, case-insensitive drag matching
- Add TC4_DELAY_CONTAINER.spec.ts (27 steps, Delay + Send Email flow)
- Add TC4/TC5/TC6 Settings & Scheduler flow specs
- Fix dragHelper.ts: case-insensitive regex matching for module names
- Fix TC2_SET_VARIABLE_CONTAINER: Done button, keep-alive polling, resilient close
- Fix TC3_DECISION_CONTAINER: try/catch for Notification/History tabs
- Fix TC1_SETTINGS_ELEMENTS: correct assertion (not.toHaveURL for history)
- Add domCapture.ts and capture_dom.ts helpers
- Update LogicContainers.xlsx with TC4 Delay test case
</commit_message>
<xml_diff>
--- a/manualtestcasedoc/LogicContainers.xlsx
+++ b/manualtestcasedoc/LogicContainers.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="143" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="154" uniqueCount="154">
   <si>
     <t>S.No</t>
   </si>
@@ -309,14 +309,14 @@
     <t>Notification section should be expanded</t>
   </si>
   <si>
-    <t>Drag and Drop the "Send Mail" action into Trigger box</t>
+    <t>Drag and Drop the "Send EMail" action into Trigger box</t>
   </si>
   <si>
-    <t>Send Mail action should be drag and dropped and SendMail popup should be opened</t>
+    <t>Send EMail action should be drag and dropped and SendMail popup should be opened</t>
   </si>
   <si>
     <r>
-      <t xml:space="preserve">Give input as </t>
+      <t xml:space="preserve">Type as </t>
     </r>
     <r>
       <t>tmaniflow@gmail.com</t>
@@ -329,7 +329,7 @@
     <t>Able to give input as mentioned</t>
   </si>
   <si>
-    <t>Give input as Automation in "Subject" field</t>
+    <t>Type as Automation in "Subject" field</t>
   </si>
   <si>
     <t>Swith ON the flow</t>
@@ -392,10 +392,16 @@
     <t>Validate the  condition in the decision container are working</t>
   </si>
   <si>
+    <t>Click DateField and set Datetime as 5 Minutes later</t>
+  </si>
+  <si>
+    <t>Able to Datetime as 5 Minutes later</t>
+  </si>
+  <si>
     <t>Give "qatest" input in "Value" field</t>
   </si>
   <si>
-    <t xml:space="preserve">Drag and Drop the "Decision" box into SetVariable action </t>
+    <t>Drag and Drop the "Decision" into Set Variable action inside canvas</t>
   </si>
   <si>
     <t>Decision box should be opened</t>
@@ -428,7 +434,7 @@
     <t>Give as "qa" value in input field</t>
   </si>
   <si>
-    <t>Drag and Drop the "Send Mail" action into the "Decision" action Direct connection</t>
+    <t>Drag and Drop the "Send EMail" action into the "Decision" action Direct connection</t>
   </si>
   <si>
     <t>Step28</t>
@@ -451,12 +457,39 @@
   <si>
     <t>Step34</t>
   </si>
+  <si>
+    <t>Delay_Container</t>
+  </si>
+  <si>
+    <t>Validate the Delay container is working</t>
+  </si>
+  <si>
+    <t>Provide FlowName as "Delayflow" in Flow Name field</t>
+  </si>
+  <si>
+    <t>Drag "Delay" into Trigger box</t>
+  </si>
+  <si>
+    <t>Drag and drop should be worked and "Delay" window opened</t>
+  </si>
+  <si>
+    <t>Give input as "1 Minute" in "Delay For"  inout field</t>
+  </si>
+  <si>
+    <t>We can able to give input in "Delay For" field</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click Delay Input </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Click Delay output </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -503,6 +536,11 @@
     </font>
     <font>
       <u/>
+      <sz val="10"/>
+      <color rgb="FF0563C1"/>
+      <name val="Arial"/>
+    </font>
+    <font>
       <sz val="10"/>
       <color rgb="FF0563C1"/>
       <name val="Arial"/>
@@ -618,7 +656,7 @@
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -675,6 +713,9 @@
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0">
       <alignment vertical="bottom"/>
+    </xf>
+    <xf borderId="4" fillId="0" fontId="11" numFmtId="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1" textRotation="0"/>
     </xf>
     <xf borderId="0" fillId="3" fontId="6" numFmtId="0" xfId="0">
       <alignment vertical="bottom" wrapText="1" textRotation="0" indent="0"/>
@@ -878,7 +919,7 @@
       <c r="Y2" s="11"/>
       <c r="Z2" s="11"/>
     </row>
-    <row r="3" ht="27.0">
+    <row r="3" customHeight="1" ht="14.0">
       <c r="A3" s="8"/>
       <c r="B3" s="8"/>
       <c r="C3" s="8"/>
@@ -913,7 +954,7 @@
       <c r="Y3" s="11"/>
       <c r="Z3" s="11"/>
     </row>
-    <row r="4" customHeight="1" ht="53.0">
+    <row r="4" customHeight="1" ht="14.0">
       <c r="A4" s="8"/>
       <c r="B4" s="8"/>
       <c r="C4" s="8"/>
@@ -948,7 +989,7 @@
       <c r="Y4" s="11"/>
       <c r="Z4" s="11"/>
     </row>
-    <row r="5" customHeight="1" ht="53.0">
+    <row r="5" customHeight="1" ht="14.0">
       <c r="A5" s="8"/>
       <c r="B5" s="8"/>
       <c r="C5" s="8"/>
@@ -983,7 +1024,7 @@
       <c r="Y5" s="11"/>
       <c r="Z5" s="11"/>
     </row>
-    <row r="6" customHeight="1" ht="53.0">
+    <row r="6" customHeight="1" ht="14.0">
       <c r="A6" s="8"/>
       <c r="B6" s="8"/>
       <c r="C6" s="8"/>
@@ -1018,7 +1059,7 @@
       <c r="Y6" s="11"/>
       <c r="Z6" s="11"/>
     </row>
-    <row r="7" customHeight="1" ht="53.0">
+    <row r="7" customHeight="1" ht="14.0">
       <c r="A7" s="8"/>
       <c r="B7" s="8"/>
       <c r="C7" s="8"/>
@@ -1053,7 +1094,7 @@
       <c r="Y7" s="11"/>
       <c r="Z7" s="11"/>
     </row>
-    <row r="8" customHeight="1" ht="53.0">
+    <row r="8" customHeight="1" ht="14.0">
       <c r="A8" s="8"/>
       <c r="B8" s="8"/>
       <c r="C8" s="8"/>
@@ -1088,7 +1129,7 @@
       <c r="Y8" s="11"/>
       <c r="Z8" s="11"/>
     </row>
-    <row r="9" customHeight="1" ht="53.0">
+    <row r="9" customHeight="1" ht="14.0">
       <c r="A9" s="8"/>
       <c r="B9" s="8"/>
       <c r="C9" s="8"/>
@@ -1123,7 +1164,7 @@
       <c r="Y9" s="11"/>
       <c r="Z9" s="11"/>
     </row>
-    <row r="10" customHeight="1" ht="53.0">
+    <row r="10" customHeight="1" ht="14.0">
       <c r="A10" s="8"/>
       <c r="B10" s="8"/>
       <c r="C10" s="8"/>
@@ -1158,7 +1199,7 @@
       <c r="Y10" s="11"/>
       <c r="Z10" s="11"/>
     </row>
-    <row r="11" customHeight="1" ht="53.0">
+    <row r="11" customHeight="1" ht="14.0">
       <c r="A11" s="8"/>
       <c r="B11" s="8"/>
       <c r="C11" s="8"/>
@@ -1193,7 +1234,7 @@
       <c r="Y11" s="11"/>
       <c r="Z11" s="11"/>
     </row>
-    <row r="12" customHeight="1" ht="53.0">
+    <row r="12" customHeight="1" ht="14.0">
       <c r="A12" s="8"/>
       <c r="B12" s="8"/>
       <c r="C12" s="8"/>
@@ -1228,7 +1269,7 @@
       <c r="Y12" s="11"/>
       <c r="Z12" s="11"/>
     </row>
-    <row r="13" customHeight="1" ht="53.0">
+    <row r="13" customHeight="1" ht="14.0">
       <c r="A13" s="8"/>
       <c r="B13" s="8"/>
       <c r="C13" s="8"/>
@@ -1263,7 +1304,7 @@
       <c r="Y13" s="11"/>
       <c r="Z13" s="11"/>
     </row>
-    <row r="14" customHeight="1" ht="53.0">
+    <row r="14" customHeight="1" ht="14.0">
       <c r="A14" s="8"/>
       <c r="B14" s="8"/>
       <c r="C14" s="8"/>
@@ -1298,7 +1339,7 @@
       <c r="Y14" s="11"/>
       <c r="Z14" s="11"/>
     </row>
-    <row r="15" customHeight="1" ht="63.0">
+    <row r="15" customHeight="1" ht="14.0">
       <c r="A15" s="8"/>
       <c r="B15" s="8"/>
       <c r="C15" s="8"/>
@@ -1333,7 +1374,7 @@
       <c r="Y15" s="11"/>
       <c r="Z15" s="11"/>
     </row>
-    <row r="16" customHeight="1" ht="63.0">
+    <row r="16" customHeight="1" ht="14.0">
       <c r="A16" s="8"/>
       <c r="B16" s="8"/>
       <c r="C16" s="8"/>
@@ -1368,7 +1409,7 @@
       <c r="Y16" s="11"/>
       <c r="Z16" s="11"/>
     </row>
-    <row r="17" customHeight="1" ht="63.0">
+    <row r="17" customHeight="1" ht="14.0">
       <c r="A17" s="8"/>
       <c r="B17" s="8"/>
       <c r="C17" s="8"/>
@@ -1403,7 +1444,7 @@
       <c r="Y17" s="11"/>
       <c r="Z17" s="11"/>
     </row>
-    <row r="18" customHeight="1" ht="63.0">
+    <row r="18" customHeight="1" ht="14.0">
       <c r="A18" s="8"/>
       <c r="B18" s="8"/>
       <c r="C18" s="8"/>
@@ -1438,7 +1479,7 @@
       <c r="Y18" s="11"/>
       <c r="Z18" s="11"/>
     </row>
-    <row r="19" customHeight="1" ht="63.0">
+    <row r="19" customHeight="1" ht="14.0">
       <c r="A19" s="8"/>
       <c r="B19" s="8"/>
       <c r="C19" s="8"/>
@@ -1473,7 +1514,7 @@
       <c r="Y19" s="11"/>
       <c r="Z19" s="11"/>
     </row>
-    <row r="20" customHeight="1" ht="63.0">
+    <row r="20" customHeight="1" ht="14.0">
       <c r="A20" s="8"/>
       <c r="B20" s="8"/>
       <c r="C20" s="8"/>
@@ -1508,7 +1549,7 @@
       <c r="Y20" s="11"/>
       <c r="Z20" s="11"/>
     </row>
-    <row r="21" customHeight="1" ht="63.0">
+    <row r="21" customHeight="1" ht="14.0">
       <c r="A21" s="8"/>
       <c r="B21" s="8"/>
       <c r="C21" s="8"/>
@@ -1543,7 +1584,7 @@
       <c r="Y21" s="11"/>
       <c r="Z21" s="11"/>
     </row>
-    <row r="22" customHeight="1" ht="63.0">
+    <row r="22" customHeight="1" ht="14.0">
       <c r="A22" s="8"/>
       <c r="B22" s="8"/>
       <c r="C22" s="8"/>
@@ -1578,7 +1619,7 @@
       <c r="Y22" s="11"/>
       <c r="Z22" s="11"/>
     </row>
-    <row r="23" customHeight="1" ht="63.0">
+    <row r="23" customHeight="1" ht="14.0">
       <c r="A23" s="8"/>
       <c r="B23" s="8"/>
       <c r="C23" s="8"/>
@@ -1613,7 +1654,7 @@
       <c r="Y23" s="11"/>
       <c r="Z23" s="11"/>
     </row>
-    <row r="24" customHeight="1" ht="63.0">
+    <row r="24" customHeight="1" ht="14.0">
       <c r="A24" s="8"/>
       <c r="B24" s="8"/>
       <c r="C24" s="8"/>
@@ -1648,7 +1689,7 @@
       <c r="Y24" s="11"/>
       <c r="Z24" s="11"/>
     </row>
-    <row r="25" customHeight="1" ht="63.0">
+    <row r="25" customHeight="1" ht="14.0">
       <c r="A25" s="8"/>
       <c r="B25" s="8"/>
       <c r="C25" s="8"/>
@@ -1683,7 +1724,7 @@
       <c r="Y25" s="11"/>
       <c r="Z25" s="11"/>
     </row>
-    <row r="26" customHeight="1" ht="63.0">
+    <row r="26" customHeight="1" ht="14.0">
       <c r="A26" s="8"/>
       <c r="B26" s="8"/>
       <c r="C26" s="8"/>
@@ -1718,7 +1759,7 @@
       <c r="Y26" s="11"/>
       <c r="Z26" s="11"/>
     </row>
-    <row r="27" customHeight="1" ht="63.0">
+    <row r="27" customHeight="1" ht="14.0">
       <c r="A27" s="8"/>
       <c r="B27" s="8"/>
       <c r="C27" s="8"/>
@@ -3155,10 +3196,10 @@
         <v>32</v>
       </c>
       <c r="F63" s="14" t="s">
-        <v>33</v>
+        <v>123</v>
       </c>
       <c r="G63" s="13" t="s">
-        <v>34</v>
+        <v>124</v>
       </c>
       <c r="H63" s="8"/>
       <c r="I63" s="10"/>
@@ -3527,7 +3568,7 @@
         <v>50</v>
       </c>
       <c r="F69" s="8" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="G69" s="9" t="s">
         <v>95</v>
@@ -3651,10 +3692,10 @@
         <v>56</v>
       </c>
       <c r="F71" s="15" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G71" s="16" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="H71" s="8"/>
       <c r="I71" s="10"/>
@@ -3713,10 +3754,10 @@
         <v>59</v>
       </c>
       <c r="F72" s="15" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G72" s="16" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="H72" s="8"/>
       <c r="I72" s="10"/>
@@ -3775,10 +3816,10 @@
         <v>62</v>
       </c>
       <c r="F73" s="15" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G73" s="16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="H73" s="8"/>
       <c r="I73" s="10"/>
@@ -3837,10 +3878,10 @@
         <v>65</v>
       </c>
       <c r="F74" s="15" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G74" s="16" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="H74" s="8"/>
       <c r="I74" s="10"/>
@@ -3899,10 +3940,10 @@
         <v>68</v>
       </c>
       <c r="F75" s="15" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G75" s="16" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="H75" s="8"/>
       <c r="I75" s="10"/>
@@ -3961,7 +4002,7 @@
         <v>71</v>
       </c>
       <c r="F76" s="15" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G76" s="16" t="s">
         <v>95</v>
@@ -4147,7 +4188,7 @@
         <v>80</v>
       </c>
       <c r="F79" s="15" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G79" s="16" t="s">
         <v>99</v>
@@ -4454,7 +4495,7 @@
         <v>13</v>
       </c>
       <c r="E84" s="12" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F84" s="8" t="s">
         <v>105</v>
@@ -4516,7 +4557,7 @@
         <v>13</v>
       </c>
       <c r="E85" s="12" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="F85" s="8" t="s">
         <v>107</v>
@@ -4578,7 +4619,7 @@
         <v>13</v>
       </c>
       <c r="E86" s="12" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F86" s="8" t="s">
         <v>109</v>
@@ -4640,7 +4681,7 @@
         <v>13</v>
       </c>
       <c r="E87" s="12" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="F87" s="8" t="s">
         <v>111</v>
@@ -4702,7 +4743,7 @@
         <v>13</v>
       </c>
       <c r="E88" s="12" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F88" s="8" t="s">
         <v>113</v>
@@ -4764,7 +4805,7 @@
         <v>13</v>
       </c>
       <c r="E89" s="12" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="F89" s="8" t="s">
         <v>116</v>
@@ -4826,7 +4867,7 @@
         <v>13</v>
       </c>
       <c r="E90" s="12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F90" s="8" t="s">
         <v>119</v>
@@ -4880,16 +4921,25 @@
       <c r="AY90" s="1"/>
       <c r="AZ90" s="1"/>
     </row>
-    <row r="91" ht="14.0">
-      <c r="A91" s="8"/>
-      <c r="B91" s="8"/>
-      <c r="C91" s="8"/>
-      <c r="D91" s="8"/>
+    <row r="91" ht="14.0" customFormat="1" s="18">
+      <c r="A91" s="8">
+        <v>4.0</v>
+      </c>
+      <c r="B91" s="8" t="s">
+        <v>145</v>
+      </c>
+      <c r="C91" s="8" t="s">
+        <v>146</v>
+      </c>
+      <c r="D91" s="12" t="s">
+        <v>11</v>
+      </c>
       <c r="E91" s="12"/>
       <c r="F91" s="8"/>
       <c r="G91" s="9"/>
       <c r="H91" s="8"/>
       <c r="I91" s="10"/>
+      <c r="J91" s="1"/>
       <c r="K91" s="11"/>
       <c r="L91" s="11"/>
       <c r="M91" s="11"/>
@@ -4906,18 +4956,52 @@
       <c r="X91" s="11"/>
       <c r="Y91" s="11"/>
       <c r="Z91" s="11"/>
-    </row>
-    <row r="92" ht="14.0">
-      <c r="A92" s="11"/>
-      <c r="B92" s="11"/>
-      <c r="C92" s="11"/>
-      <c r="D92" s="11"/>
-      <c r="E92" s="11"/>
-      <c r="F92" s="11"/>
-      <c r="G92" s="11"/>
-      <c r="H92" s="11"/>
-      <c r="I92" s="11"/>
-      <c r="J92" s="11"/>
+      <c r="AA91" s="1"/>
+      <c r="AB91" s="1"/>
+      <c r="AC91" s="1"/>
+      <c r="AD91" s="1"/>
+      <c r="AE91" s="1"/>
+      <c r="AF91" s="1"/>
+      <c r="AG91" s="1"/>
+      <c r="AH91" s="1"/>
+      <c r="AI91" s="1"/>
+      <c r="AJ91" s="1"/>
+      <c r="AK91" s="1"/>
+      <c r="AL91" s="1"/>
+      <c r="AM91" s="1"/>
+      <c r="AN91" s="1"/>
+      <c r="AO91" s="1"/>
+      <c r="AP91" s="1"/>
+      <c r="AQ91" s="1"/>
+      <c r="AR91" s="1"/>
+      <c r="AS91" s="1"/>
+      <c r="AT91" s="1"/>
+      <c r="AU91" s="1"/>
+      <c r="AV91" s="1"/>
+      <c r="AW91" s="1"/>
+      <c r="AX91" s="1"/>
+      <c r="AY91" s="1"/>
+      <c r="AZ91" s="1"/>
+    </row>
+    <row r="92" ht="14.0" customFormat="1" s="18">
+      <c r="A92" s="8"/>
+      <c r="B92" s="8"/>
+      <c r="C92" s="8"/>
+      <c r="D92" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E92" s="12" t="s">
+        <v>14</v>
+      </c>
+      <c r="F92" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="G92" s="9" t="s">
+        <v>16</v>
+      </c>
+      <c r="H92" s="8"/>
+      <c r="I92" s="10"/>
+      <c r="J92" s="1"/>
       <c r="K92" s="11"/>
       <c r="L92" s="11"/>
       <c r="M92" s="11"/>
@@ -4934,18 +5018,52 @@
       <c r="X92" s="11"/>
       <c r="Y92" s="11"/>
       <c r="Z92" s="11"/>
-    </row>
-    <row r="93" ht="14.0">
-      <c r="A93" s="11"/>
-      <c r="B93" s="11"/>
-      <c r="C93" s="11"/>
-      <c r="D93" s="11"/>
-      <c r="E93" s="11"/>
-      <c r="F93" s="11"/>
-      <c r="G93" s="11"/>
-      <c r="H93" s="11"/>
-      <c r="I93" s="11"/>
-      <c r="J93" s="11"/>
+      <c r="AA92" s="1"/>
+      <c r="AB92" s="1"/>
+      <c r="AC92" s="1"/>
+      <c r="AD92" s="1"/>
+      <c r="AE92" s="1"/>
+      <c r="AF92" s="1"/>
+      <c r="AG92" s="1"/>
+      <c r="AH92" s="1"/>
+      <c r="AI92" s="1"/>
+      <c r="AJ92" s="1"/>
+      <c r="AK92" s="1"/>
+      <c r="AL92" s="1"/>
+      <c r="AM92" s="1"/>
+      <c r="AN92" s="1"/>
+      <c r="AO92" s="1"/>
+      <c r="AP92" s="1"/>
+      <c r="AQ92" s="1"/>
+      <c r="AR92" s="1"/>
+      <c r="AS92" s="1"/>
+      <c r="AT92" s="1"/>
+      <c r="AU92" s="1"/>
+      <c r="AV92" s="1"/>
+      <c r="AW92" s="1"/>
+      <c r="AX92" s="1"/>
+      <c r="AY92" s="1"/>
+      <c r="AZ92" s="1"/>
+    </row>
+    <row r="93" ht="14.0" customFormat="1" s="18">
+      <c r="A93" s="8"/>
+      <c r="B93" s="8"/>
+      <c r="C93" s="8"/>
+      <c r="D93" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E93" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F93" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="G93" s="9" t="s">
+        <v>19</v>
+      </c>
+      <c r="H93" s="8"/>
+      <c r="I93" s="10"/>
+      <c r="J93" s="1"/>
       <c r="K93" s="11"/>
       <c r="L93" s="11"/>
       <c r="M93" s="11"/>
@@ -4962,18 +5080,52 @@
       <c r="X93" s="11"/>
       <c r="Y93" s="11"/>
       <c r="Z93" s="11"/>
-    </row>
-    <row r="94" ht="14.0">
-      <c r="A94" s="11"/>
-      <c r="B94" s="11"/>
-      <c r="C94" s="11"/>
-      <c r="D94" s="11"/>
-      <c r="E94" s="11"/>
-      <c r="F94" s="11"/>
-      <c r="G94" s="11"/>
-      <c r="H94" s="11"/>
-      <c r="I94" s="11"/>
-      <c r="J94" s="11"/>
+      <c r="AA93" s="1"/>
+      <c r="AB93" s="1"/>
+      <c r="AC93" s="1"/>
+      <c r="AD93" s="1"/>
+      <c r="AE93" s="1"/>
+      <c r="AF93" s="1"/>
+      <c r="AG93" s="1"/>
+      <c r="AH93" s="1"/>
+      <c r="AI93" s="1"/>
+      <c r="AJ93" s="1"/>
+      <c r="AK93" s="1"/>
+      <c r="AL93" s="1"/>
+      <c r="AM93" s="1"/>
+      <c r="AN93" s="1"/>
+      <c r="AO93" s="1"/>
+      <c r="AP93" s="1"/>
+      <c r="AQ93" s="1"/>
+      <c r="AR93" s="1"/>
+      <c r="AS93" s="1"/>
+      <c r="AT93" s="1"/>
+      <c r="AU93" s="1"/>
+      <c r="AV93" s="1"/>
+      <c r="AW93" s="1"/>
+      <c r="AX93" s="1"/>
+      <c r="AY93" s="1"/>
+      <c r="AZ93" s="1"/>
+    </row>
+    <row r="94" ht="14.0" customFormat="1" s="18">
+      <c r="A94" s="8"/>
+      <c r="B94" s="8"/>
+      <c r="C94" s="8"/>
+      <c r="D94" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E94" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="F94" s="8" t="s">
+        <v>147</v>
+      </c>
+      <c r="G94" s="9" t="s">
+        <v>22</v>
+      </c>
+      <c r="H94" s="8"/>
+      <c r="I94" s="10"/>
+      <c r="J94" s="1"/>
       <c r="K94" s="11"/>
       <c r="L94" s="11"/>
       <c r="M94" s="11"/>
@@ -4990,18 +5142,52 @@
       <c r="X94" s="11"/>
       <c r="Y94" s="11"/>
       <c r="Z94" s="11"/>
-    </row>
-    <row r="95" ht="14.0">
-      <c r="A95" s="11"/>
-      <c r="B95" s="11"/>
-      <c r="C95" s="11"/>
-      <c r="D95" s="11"/>
-      <c r="E95" s="11"/>
-      <c r="F95" s="11"/>
-      <c r="G95" s="11"/>
-      <c r="H95" s="11"/>
-      <c r="I95" s="11"/>
-      <c r="J95" s="11"/>
+      <c r="AA94" s="1"/>
+      <c r="AB94" s="1"/>
+      <c r="AC94" s="1"/>
+      <c r="AD94" s="1"/>
+      <c r="AE94" s="1"/>
+      <c r="AF94" s="1"/>
+      <c r="AG94" s="1"/>
+      <c r="AH94" s="1"/>
+      <c r="AI94" s="1"/>
+      <c r="AJ94" s="1"/>
+      <c r="AK94" s="1"/>
+      <c r="AL94" s="1"/>
+      <c r="AM94" s="1"/>
+      <c r="AN94" s="1"/>
+      <c r="AO94" s="1"/>
+      <c r="AP94" s="1"/>
+      <c r="AQ94" s="1"/>
+      <c r="AR94" s="1"/>
+      <c r="AS94" s="1"/>
+      <c r="AT94" s="1"/>
+      <c r="AU94" s="1"/>
+      <c r="AV94" s="1"/>
+      <c r="AW94" s="1"/>
+      <c r="AX94" s="1"/>
+      <c r="AY94" s="1"/>
+      <c r="AZ94" s="1"/>
+    </row>
+    <row r="95" ht="14.0" customFormat="1" s="18">
+      <c r="A95" s="8"/>
+      <c r="B95" s="8"/>
+      <c r="C95" s="8"/>
+      <c r="D95" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E95" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="F95" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="G95" s="9" t="s">
+        <v>25</v>
+      </c>
+      <c r="H95" s="8"/>
+      <c r="I95" s="10"/>
+      <c r="J95" s="1"/>
       <c r="K95" s="11"/>
       <c r="L95" s="11"/>
       <c r="M95" s="11"/>
@@ -5018,18 +5204,52 @@
       <c r="X95" s="11"/>
       <c r="Y95" s="11"/>
       <c r="Z95" s="11"/>
-    </row>
-    <row r="96" ht="14.0">
-      <c r="A96" s="11"/>
-      <c r="B96" s="11"/>
-      <c r="C96" s="11"/>
-      <c r="D96" s="11"/>
-      <c r="E96" s="11"/>
-      <c r="F96" s="11"/>
-      <c r="G96" s="11"/>
-      <c r="H96" s="11"/>
-      <c r="I96" s="11"/>
-      <c r="J96" s="11"/>
+      <c r="AA95" s="1"/>
+      <c r="AB95" s="1"/>
+      <c r="AC95" s="1"/>
+      <c r="AD95" s="1"/>
+      <c r="AE95" s="1"/>
+      <c r="AF95" s="1"/>
+      <c r="AG95" s="1"/>
+      <c r="AH95" s="1"/>
+      <c r="AI95" s="1"/>
+      <c r="AJ95" s="1"/>
+      <c r="AK95" s="1"/>
+      <c r="AL95" s="1"/>
+      <c r="AM95" s="1"/>
+      <c r="AN95" s="1"/>
+      <c r="AO95" s="1"/>
+      <c r="AP95" s="1"/>
+      <c r="AQ95" s="1"/>
+      <c r="AR95" s="1"/>
+      <c r="AS95" s="1"/>
+      <c r="AT95" s="1"/>
+      <c r="AU95" s="1"/>
+      <c r="AV95" s="1"/>
+      <c r="AW95" s="1"/>
+      <c r="AX95" s="1"/>
+      <c r="AY95" s="1"/>
+      <c r="AZ95" s="1"/>
+    </row>
+    <row r="96" ht="14.0" customFormat="1" s="18">
+      <c r="A96" s="8"/>
+      <c r="B96" s="8"/>
+      <c r="C96" s="8"/>
+      <c r="D96" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E96" s="12" t="s">
+        <v>26</v>
+      </c>
+      <c r="F96" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="G96" s="9" t="s">
+        <v>28</v>
+      </c>
+      <c r="H96" s="8"/>
+      <c r="I96" s="10"/>
+      <c r="J96" s="1"/>
       <c r="K96" s="11"/>
       <c r="L96" s="11"/>
       <c r="M96" s="11"/>
@@ -5046,18 +5266,52 @@
       <c r="X96" s="11"/>
       <c r="Y96" s="11"/>
       <c r="Z96" s="11"/>
-    </row>
-    <row r="97" ht="14.0">
-      <c r="A97" s="11"/>
-      <c r="B97" s="11"/>
-      <c r="C97" s="11"/>
-      <c r="D97" s="11"/>
-      <c r="E97" s="11"/>
-      <c r="F97" s="11"/>
-      <c r="G97" s="11"/>
-      <c r="H97" s="11"/>
-      <c r="I97" s="11"/>
-      <c r="J97" s="11"/>
+      <c r="AA96" s="1"/>
+      <c r="AB96" s="1"/>
+      <c r="AC96" s="1"/>
+      <c r="AD96" s="1"/>
+      <c r="AE96" s="1"/>
+      <c r="AF96" s="1"/>
+      <c r="AG96" s="1"/>
+      <c r="AH96" s="1"/>
+      <c r="AI96" s="1"/>
+      <c r="AJ96" s="1"/>
+      <c r="AK96" s="1"/>
+      <c r="AL96" s="1"/>
+      <c r="AM96" s="1"/>
+      <c r="AN96" s="1"/>
+      <c r="AO96" s="1"/>
+      <c r="AP96" s="1"/>
+      <c r="AQ96" s="1"/>
+      <c r="AR96" s="1"/>
+      <c r="AS96" s="1"/>
+      <c r="AT96" s="1"/>
+      <c r="AU96" s="1"/>
+      <c r="AV96" s="1"/>
+      <c r="AW96" s="1"/>
+      <c r="AX96" s="1"/>
+      <c r="AY96" s="1"/>
+      <c r="AZ96" s="1"/>
+    </row>
+    <row r="97" ht="14.0" customFormat="1" s="18">
+      <c r="A97" s="8"/>
+      <c r="B97" s="8"/>
+      <c r="C97" s="8"/>
+      <c r="D97" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E97" s="12" t="s">
+        <v>29</v>
+      </c>
+      <c r="F97" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="G97" s="9" t="s">
+        <v>31</v>
+      </c>
+      <c r="H97" s="8"/>
+      <c r="I97" s="10"/>
+      <c r="J97" s="1"/>
       <c r="K97" s="11"/>
       <c r="L97" s="11"/>
       <c r="M97" s="11"/>
@@ -5074,18 +5328,52 @@
       <c r="X97" s="11"/>
       <c r="Y97" s="11"/>
       <c r="Z97" s="11"/>
-    </row>
-    <row r="98" ht="14.0">
-      <c r="A98" s="11"/>
-      <c r="B98" s="11"/>
-      <c r="C98" s="11"/>
-      <c r="D98" s="11"/>
-      <c r="E98" s="11"/>
-      <c r="F98" s="11"/>
-      <c r="G98" s="11"/>
-      <c r="H98" s="11"/>
-      <c r="I98" s="11"/>
-      <c r="J98" s="11"/>
+      <c r="AA97" s="1"/>
+      <c r="AB97" s="1"/>
+      <c r="AC97" s="1"/>
+      <c r="AD97" s="1"/>
+      <c r="AE97" s="1"/>
+      <c r="AF97" s="1"/>
+      <c r="AG97" s="1"/>
+      <c r="AH97" s="1"/>
+      <c r="AI97" s="1"/>
+      <c r="AJ97" s="1"/>
+      <c r="AK97" s="1"/>
+      <c r="AL97" s="1"/>
+      <c r="AM97" s="1"/>
+      <c r="AN97" s="1"/>
+      <c r="AO97" s="1"/>
+      <c r="AP97" s="1"/>
+      <c r="AQ97" s="1"/>
+      <c r="AR97" s="1"/>
+      <c r="AS97" s="1"/>
+      <c r="AT97" s="1"/>
+      <c r="AU97" s="1"/>
+      <c r="AV97" s="1"/>
+      <c r="AW97" s="1"/>
+      <c r="AX97" s="1"/>
+      <c r="AY97" s="1"/>
+      <c r="AZ97" s="1"/>
+    </row>
+    <row r="98" ht="14.0" customFormat="1" s="18">
+      <c r="A98" s="8"/>
+      <c r="B98" s="8"/>
+      <c r="C98" s="8"/>
+      <c r="D98" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E98" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="F98" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="G98" s="9" t="s">
+        <v>34</v>
+      </c>
+      <c r="H98" s="8"/>
+      <c r="I98" s="10"/>
+      <c r="J98" s="1"/>
       <c r="K98" s="11"/>
       <c r="L98" s="11"/>
       <c r="M98" s="11"/>
@@ -5102,18 +5390,52 @@
       <c r="X98" s="11"/>
       <c r="Y98" s="11"/>
       <c r="Z98" s="11"/>
-    </row>
-    <row r="99" ht="14.0">
-      <c r="A99" s="11"/>
-      <c r="B99" s="11"/>
-      <c r="C99" s="11"/>
-      <c r="D99" s="11"/>
-      <c r="E99" s="11"/>
-      <c r="F99" s="11"/>
-      <c r="G99" s="11"/>
-      <c r="H99" s="11"/>
-      <c r="I99" s="11"/>
-      <c r="J99" s="11"/>
+      <c r="AA98" s="1"/>
+      <c r="AB98" s="1"/>
+      <c r="AC98" s="1"/>
+      <c r="AD98" s="1"/>
+      <c r="AE98" s="1"/>
+      <c r="AF98" s="1"/>
+      <c r="AG98" s="1"/>
+      <c r="AH98" s="1"/>
+      <c r="AI98" s="1"/>
+      <c r="AJ98" s="1"/>
+      <c r="AK98" s="1"/>
+      <c r="AL98" s="1"/>
+      <c r="AM98" s="1"/>
+      <c r="AN98" s="1"/>
+      <c r="AO98" s="1"/>
+      <c r="AP98" s="1"/>
+      <c r="AQ98" s="1"/>
+      <c r="AR98" s="1"/>
+      <c r="AS98" s="1"/>
+      <c r="AT98" s="1"/>
+      <c r="AU98" s="1"/>
+      <c r="AV98" s="1"/>
+      <c r="AW98" s="1"/>
+      <c r="AX98" s="1"/>
+      <c r="AY98" s="1"/>
+      <c r="AZ98" s="1"/>
+    </row>
+    <row r="99" ht="14.0" customFormat="1" s="18">
+      <c r="A99" s="8"/>
+      <c r="B99" s="8"/>
+      <c r="C99" s="8"/>
+      <c r="D99" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E99" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F99" s="8" t="s">
+        <v>36</v>
+      </c>
+      <c r="G99" s="9" t="s">
+        <v>37</v>
+      </c>
+      <c r="H99" s="8"/>
+      <c r="I99" s="10"/>
+      <c r="J99" s="1"/>
       <c r="K99" s="11"/>
       <c r="L99" s="11"/>
       <c r="M99" s="11"/>
@@ -5130,18 +5452,52 @@
       <c r="X99" s="11"/>
       <c r="Y99" s="11"/>
       <c r="Z99" s="11"/>
-    </row>
-    <row r="100" ht="14.0">
-      <c r="A100" s="11"/>
-      <c r="B100" s="11"/>
-      <c r="C100" s="11"/>
-      <c r="D100" s="11"/>
-      <c r="E100" s="11"/>
-      <c r="F100" s="11"/>
-      <c r="G100" s="11"/>
-      <c r="H100" s="11"/>
-      <c r="I100" s="11"/>
-      <c r="J100" s="11"/>
+      <c r="AA99" s="1"/>
+      <c r="AB99" s="1"/>
+      <c r="AC99" s="1"/>
+      <c r="AD99" s="1"/>
+      <c r="AE99" s="1"/>
+      <c r="AF99" s="1"/>
+      <c r="AG99" s="1"/>
+      <c r="AH99" s="1"/>
+      <c r="AI99" s="1"/>
+      <c r="AJ99" s="1"/>
+      <c r="AK99" s="1"/>
+      <c r="AL99" s="1"/>
+      <c r="AM99" s="1"/>
+      <c r="AN99" s="1"/>
+      <c r="AO99" s="1"/>
+      <c r="AP99" s="1"/>
+      <c r="AQ99" s="1"/>
+      <c r="AR99" s="1"/>
+      <c r="AS99" s="1"/>
+      <c r="AT99" s="1"/>
+      <c r="AU99" s="1"/>
+      <c r="AV99" s="1"/>
+      <c r="AW99" s="1"/>
+      <c r="AX99" s="1"/>
+      <c r="AY99" s="1"/>
+      <c r="AZ99" s="1"/>
+    </row>
+    <row r="100" ht="14.0" customFormat="1" s="18">
+      <c r="A100" s="8"/>
+      <c r="B100" s="8"/>
+      <c r="C100" s="8"/>
+      <c r="D100" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E100" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="F100" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G100" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H100" s="8"/>
+      <c r="I100" s="10"/>
+      <c r="J100" s="1"/>
       <c r="K100" s="11"/>
       <c r="L100" s="11"/>
       <c r="M100" s="11"/>
@@ -5158,18 +5514,52 @@
       <c r="X100" s="11"/>
       <c r="Y100" s="11"/>
       <c r="Z100" s="11"/>
-    </row>
-    <row r="101" ht="14.0">
-      <c r="A101" s="11"/>
-      <c r="B101" s="11"/>
-      <c r="C101" s="11"/>
-      <c r="D101" s="11"/>
-      <c r="E101" s="11"/>
-      <c r="F101" s="11"/>
-      <c r="G101" s="11"/>
-      <c r="H101" s="11"/>
-      <c r="I101" s="11"/>
-      <c r="J101" s="11"/>
+      <c r="AA100" s="1"/>
+      <c r="AB100" s="1"/>
+      <c r="AC100" s="1"/>
+      <c r="AD100" s="1"/>
+      <c r="AE100" s="1"/>
+      <c r="AF100" s="1"/>
+      <c r="AG100" s="1"/>
+      <c r="AH100" s="1"/>
+      <c r="AI100" s="1"/>
+      <c r="AJ100" s="1"/>
+      <c r="AK100" s="1"/>
+      <c r="AL100" s="1"/>
+      <c r="AM100" s="1"/>
+      <c r="AN100" s="1"/>
+      <c r="AO100" s="1"/>
+      <c r="AP100" s="1"/>
+      <c r="AQ100" s="1"/>
+      <c r="AR100" s="1"/>
+      <c r="AS100" s="1"/>
+      <c r="AT100" s="1"/>
+      <c r="AU100" s="1"/>
+      <c r="AV100" s="1"/>
+      <c r="AW100" s="1"/>
+      <c r="AX100" s="1"/>
+      <c r="AY100" s="1"/>
+      <c r="AZ100" s="1"/>
+    </row>
+    <row r="101" ht="14.0" customFormat="1" s="18">
+      <c r="A101" s="8"/>
+      <c r="B101" s="8"/>
+      <c r="C101" s="8"/>
+      <c r="D101" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E101" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="F101" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="G101" s="9" t="s">
+        <v>91</v>
+      </c>
+      <c r="H101" s="8"/>
+      <c r="I101" s="10"/>
+      <c r="J101" s="1"/>
       <c r="K101" s="11"/>
       <c r="L101" s="11"/>
       <c r="M101" s="11"/>
@@ -5186,18 +5576,52 @@
       <c r="X101" s="11"/>
       <c r="Y101" s="11"/>
       <c r="Z101" s="11"/>
-    </row>
-    <row r="102" ht="14.0">
-      <c r="A102" s="11"/>
-      <c r="B102" s="11"/>
-      <c r="C102" s="11"/>
-      <c r="D102" s="11"/>
-      <c r="E102" s="11"/>
-      <c r="F102" s="11"/>
-      <c r="G102" s="11"/>
-      <c r="H102" s="11"/>
-      <c r="I102" s="11"/>
-      <c r="J102" s="11"/>
+      <c r="AA101" s="1"/>
+      <c r="AB101" s="1"/>
+      <c r="AC101" s="1"/>
+      <c r="AD101" s="1"/>
+      <c r="AE101" s="1"/>
+      <c r="AF101" s="1"/>
+      <c r="AG101" s="1"/>
+      <c r="AH101" s="1"/>
+      <c r="AI101" s="1"/>
+      <c r="AJ101" s="1"/>
+      <c r="AK101" s="1"/>
+      <c r="AL101" s="1"/>
+      <c r="AM101" s="1"/>
+      <c r="AN101" s="1"/>
+      <c r="AO101" s="1"/>
+      <c r="AP101" s="1"/>
+      <c r="AQ101" s="1"/>
+      <c r="AR101" s="1"/>
+      <c r="AS101" s="1"/>
+      <c r="AT101" s="1"/>
+      <c r="AU101" s="1"/>
+      <c r="AV101" s="1"/>
+      <c r="AW101" s="1"/>
+      <c r="AX101" s="1"/>
+      <c r="AY101" s="1"/>
+      <c r="AZ101" s="1"/>
+    </row>
+    <row r="102" ht="14.0" customFormat="1" s="18">
+      <c r="A102" s="8"/>
+      <c r="B102" s="8"/>
+      <c r="C102" s="8"/>
+      <c r="D102" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E102" s="12" t="s">
+        <v>44</v>
+      </c>
+      <c r="F102" s="8" t="s">
+        <v>45</v>
+      </c>
+      <c r="G102" s="9" t="s">
+        <v>46</v>
+      </c>
+      <c r="H102" s="8"/>
+      <c r="I102" s="10"/>
+      <c r="J102" s="1"/>
       <c r="K102" s="11"/>
       <c r="L102" s="11"/>
       <c r="M102" s="11"/>
@@ -5214,18 +5638,52 @@
       <c r="X102" s="11"/>
       <c r="Y102" s="11"/>
       <c r="Z102" s="11"/>
-    </row>
-    <row r="103" ht="14.0">
-      <c r="A103" s="11"/>
-      <c r="B103" s="11"/>
-      <c r="C103" s="11"/>
-      <c r="D103" s="11"/>
-      <c r="E103" s="11"/>
-      <c r="F103" s="11"/>
-      <c r="G103" s="11"/>
-      <c r="H103" s="11"/>
-      <c r="I103" s="11"/>
-      <c r="J103" s="11"/>
+      <c r="AA102" s="1"/>
+      <c r="AB102" s="1"/>
+      <c r="AC102" s="1"/>
+      <c r="AD102" s="1"/>
+      <c r="AE102" s="1"/>
+      <c r="AF102" s="1"/>
+      <c r="AG102" s="1"/>
+      <c r="AH102" s="1"/>
+      <c r="AI102" s="1"/>
+      <c r="AJ102" s="1"/>
+      <c r="AK102" s="1"/>
+      <c r="AL102" s="1"/>
+      <c r="AM102" s="1"/>
+      <c r="AN102" s="1"/>
+      <c r="AO102" s="1"/>
+      <c r="AP102" s="1"/>
+      <c r="AQ102" s="1"/>
+      <c r="AR102" s="1"/>
+      <c r="AS102" s="1"/>
+      <c r="AT102" s="1"/>
+      <c r="AU102" s="1"/>
+      <c r="AV102" s="1"/>
+      <c r="AW102" s="1"/>
+      <c r="AX102" s="1"/>
+      <c r="AY102" s="1"/>
+      <c r="AZ102" s="1"/>
+    </row>
+    <row r="103" ht="27.0" customFormat="1" s="18">
+      <c r="A103" s="8"/>
+      <c r="B103" s="8"/>
+      <c r="C103" s="8"/>
+      <c r="D103" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E103" s="12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F103" s="8" t="s">
+        <v>148</v>
+      </c>
+      <c r="G103" s="9" t="s">
+        <v>149</v>
+      </c>
+      <c r="H103" s="8"/>
+      <c r="I103" s="10"/>
+      <c r="J103" s="1"/>
       <c r="K103" s="11"/>
       <c r="L103" s="11"/>
       <c r="M103" s="11"/>
@@ -5242,18 +5700,52 @@
       <c r="X103" s="11"/>
       <c r="Y103" s="11"/>
       <c r="Z103" s="11"/>
-    </row>
-    <row r="104" ht="14.0">
-      <c r="A104" s="11"/>
-      <c r="B104" s="11"/>
-      <c r="C104" s="11"/>
-      <c r="D104" s="11"/>
-      <c r="E104" s="11"/>
-      <c r="F104" s="11"/>
-      <c r="G104" s="11"/>
-      <c r="H104" s="11"/>
-      <c r="I104" s="11"/>
-      <c r="J104" s="11"/>
+      <c r="AA103" s="1"/>
+      <c r="AB103" s="1"/>
+      <c r="AC103" s="1"/>
+      <c r="AD103" s="1"/>
+      <c r="AE103" s="1"/>
+      <c r="AF103" s="1"/>
+      <c r="AG103" s="1"/>
+      <c r="AH103" s="1"/>
+      <c r="AI103" s="1"/>
+      <c r="AJ103" s="1"/>
+      <c r="AK103" s="1"/>
+      <c r="AL103" s="1"/>
+      <c r="AM103" s="1"/>
+      <c r="AN103" s="1"/>
+      <c r="AO103" s="1"/>
+      <c r="AP103" s="1"/>
+      <c r="AQ103" s="1"/>
+      <c r="AR103" s="1"/>
+      <c r="AS103" s="1"/>
+      <c r="AT103" s="1"/>
+      <c r="AU103" s="1"/>
+      <c r="AV103" s="1"/>
+      <c r="AW103" s="1"/>
+      <c r="AX103" s="1"/>
+      <c r="AY103" s="1"/>
+      <c r="AZ103" s="1"/>
+    </row>
+    <row r="104" ht="27.0" customFormat="1" s="18">
+      <c r="A104" s="8"/>
+      <c r="B104" s="8"/>
+      <c r="C104" s="8"/>
+      <c r="D104" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E104" s="12" t="s">
+        <v>50</v>
+      </c>
+      <c r="F104" s="8" t="s">
+        <v>150</v>
+      </c>
+      <c r="G104" s="9" t="s">
+        <v>151</v>
+      </c>
+      <c r="H104" s="8"/>
+      <c r="I104" s="10"/>
+      <c r="J104" s="1"/>
       <c r="K104" s="11"/>
       <c r="L104" s="11"/>
       <c r="M104" s="11"/>
@@ -5270,18 +5762,52 @@
       <c r="X104" s="11"/>
       <c r="Y104" s="11"/>
       <c r="Z104" s="11"/>
-    </row>
-    <row r="105" ht="14.0">
-      <c r="A105" s="11"/>
-      <c r="B105" s="11"/>
-      <c r="C105" s="11"/>
-      <c r="D105" s="11"/>
-      <c r="E105" s="11"/>
-      <c r="F105" s="11"/>
-      <c r="G105" s="11"/>
-      <c r="H105" s="11"/>
-      <c r="I105" s="11"/>
-      <c r="J105" s="11"/>
+      <c r="AA104" s="1"/>
+      <c r="AB104" s="1"/>
+      <c r="AC104" s="1"/>
+      <c r="AD104" s="1"/>
+      <c r="AE104" s="1"/>
+      <c r="AF104" s="1"/>
+      <c r="AG104" s="1"/>
+      <c r="AH104" s="1"/>
+      <c r="AI104" s="1"/>
+      <c r="AJ104" s="1"/>
+      <c r="AK104" s="1"/>
+      <c r="AL104" s="1"/>
+      <c r="AM104" s="1"/>
+      <c r="AN104" s="1"/>
+      <c r="AO104" s="1"/>
+      <c r="AP104" s="1"/>
+      <c r="AQ104" s="1"/>
+      <c r="AR104" s="1"/>
+      <c r="AS104" s="1"/>
+      <c r="AT104" s="1"/>
+      <c r="AU104" s="1"/>
+      <c r="AV104" s="1"/>
+      <c r="AW104" s="1"/>
+      <c r="AX104" s="1"/>
+      <c r="AY104" s="1"/>
+      <c r="AZ104" s="1"/>
+    </row>
+    <row r="105" ht="14.0" customFormat="1" s="18">
+      <c r="A105" s="8"/>
+      <c r="B105" s="8"/>
+      <c r="C105" s="8"/>
+      <c r="D105" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E105" s="12" t="s">
+        <v>53</v>
+      </c>
+      <c r="F105" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G105" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H105" s="8"/>
+      <c r="I105" s="10"/>
+      <c r="J105" s="1"/>
       <c r="K105" s="11"/>
       <c r="L105" s="11"/>
       <c r="M105" s="11"/>
@@ -5298,18 +5824,52 @@
       <c r="X105" s="11"/>
       <c r="Y105" s="11"/>
       <c r="Z105" s="11"/>
-    </row>
-    <row r="106" ht="14.0">
-      <c r="A106" s="11"/>
-      <c r="B106" s="11"/>
-      <c r="C106" s="11"/>
-      <c r="D106" s="11"/>
-      <c r="E106" s="11"/>
-      <c r="F106" s="11"/>
-      <c r="G106" s="11"/>
-      <c r="H106" s="11"/>
-      <c r="I106" s="11"/>
-      <c r="J106" s="11"/>
+      <c r="AA105" s="1"/>
+      <c r="AB105" s="1"/>
+      <c r="AC105" s="1"/>
+      <c r="AD105" s="1"/>
+      <c r="AE105" s="1"/>
+      <c r="AF105" s="1"/>
+      <c r="AG105" s="1"/>
+      <c r="AH105" s="1"/>
+      <c r="AI105" s="1"/>
+      <c r="AJ105" s="1"/>
+      <c r="AK105" s="1"/>
+      <c r="AL105" s="1"/>
+      <c r="AM105" s="1"/>
+      <c r="AN105" s="1"/>
+      <c r="AO105" s="1"/>
+      <c r="AP105" s="1"/>
+      <c r="AQ105" s="1"/>
+      <c r="AR105" s="1"/>
+      <c r="AS105" s="1"/>
+      <c r="AT105" s="1"/>
+      <c r="AU105" s="1"/>
+      <c r="AV105" s="1"/>
+      <c r="AW105" s="1"/>
+      <c r="AX105" s="1"/>
+      <c r="AY105" s="1"/>
+      <c r="AZ105" s="1"/>
+    </row>
+    <row r="106" ht="14.0" customFormat="1" s="18">
+      <c r="A106" s="8"/>
+      <c r="B106" s="8"/>
+      <c r="C106" s="8"/>
+      <c r="D106" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E106" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="F106" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="G106" s="9" t="s">
+        <v>97</v>
+      </c>
+      <c r="H106" s="8"/>
+      <c r="I106" s="10"/>
+      <c r="J106" s="1"/>
       <c r="K106" s="11"/>
       <c r="L106" s="11"/>
       <c r="M106" s="11"/>
@@ -5326,18 +5886,52 @@
       <c r="X106" s="11"/>
       <c r="Y106" s="11"/>
       <c r="Z106" s="11"/>
-    </row>
-    <row r="107" ht="14.0">
-      <c r="A107" s="11"/>
-      <c r="B107" s="11"/>
-      <c r="C107" s="11"/>
-      <c r="D107" s="11"/>
-      <c r="E107" s="11"/>
-      <c r="F107" s="11"/>
-      <c r="G107" s="11"/>
-      <c r="H107" s="11"/>
-      <c r="I107" s="11"/>
-      <c r="J107" s="11"/>
+      <c r="AA106" s="1"/>
+      <c r="AB106" s="1"/>
+      <c r="AC106" s="1"/>
+      <c r="AD106" s="1"/>
+      <c r="AE106" s="1"/>
+      <c r="AF106" s="1"/>
+      <c r="AG106" s="1"/>
+      <c r="AH106" s="1"/>
+      <c r="AI106" s="1"/>
+      <c r="AJ106" s="1"/>
+      <c r="AK106" s="1"/>
+      <c r="AL106" s="1"/>
+      <c r="AM106" s="1"/>
+      <c r="AN106" s="1"/>
+      <c r="AO106" s="1"/>
+      <c r="AP106" s="1"/>
+      <c r="AQ106" s="1"/>
+      <c r="AR106" s="1"/>
+      <c r="AS106" s="1"/>
+      <c r="AT106" s="1"/>
+      <c r="AU106" s="1"/>
+      <c r="AV106" s="1"/>
+      <c r="AW106" s="1"/>
+      <c r="AX106" s="1"/>
+      <c r="AY106" s="1"/>
+      <c r="AZ106" s="1"/>
+    </row>
+    <row r="107" ht="41.0" customFormat="1" s="18">
+      <c r="A107" s="8"/>
+      <c r="B107" s="8"/>
+      <c r="C107" s="8"/>
+      <c r="D107" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E107" s="12" t="s">
+        <v>59</v>
+      </c>
+      <c r="F107" s="8" t="s">
+        <v>98</v>
+      </c>
+      <c r="G107" s="9" t="s">
+        <v>99</v>
+      </c>
+      <c r="H107" s="8"/>
+      <c r="I107" s="10"/>
+      <c r="J107" s="1"/>
       <c r="K107" s="11"/>
       <c r="L107" s="11"/>
       <c r="M107" s="11"/>
@@ -5354,18 +5948,52 @@
       <c r="X107" s="11"/>
       <c r="Y107" s="11"/>
       <c r="Z107" s="11"/>
-    </row>
-    <row r="108" ht="14.0">
-      <c r="A108" s="11"/>
-      <c r="B108" s="11"/>
-      <c r="C108" s="11"/>
-      <c r="D108" s="11"/>
-      <c r="E108" s="11"/>
-      <c r="F108" s="11"/>
-      <c r="G108" s="11"/>
-      <c r="H108" s="11"/>
-      <c r="I108" s="11"/>
-      <c r="J108" s="11"/>
+      <c r="AA107" s="1"/>
+      <c r="AB107" s="1"/>
+      <c r="AC107" s="1"/>
+      <c r="AD107" s="1"/>
+      <c r="AE107" s="1"/>
+      <c r="AF107" s="1"/>
+      <c r="AG107" s="1"/>
+      <c r="AH107" s="1"/>
+      <c r="AI107" s="1"/>
+      <c r="AJ107" s="1"/>
+      <c r="AK107" s="1"/>
+      <c r="AL107" s="1"/>
+      <c r="AM107" s="1"/>
+      <c r="AN107" s="1"/>
+      <c r="AO107" s="1"/>
+      <c r="AP107" s="1"/>
+      <c r="AQ107" s="1"/>
+      <c r="AR107" s="1"/>
+      <c r="AS107" s="1"/>
+      <c r="AT107" s="1"/>
+      <c r="AU107" s="1"/>
+      <c r="AV107" s="1"/>
+      <c r="AW107" s="1"/>
+      <c r="AX107" s="1"/>
+      <c r="AY107" s="1"/>
+      <c r="AZ107" s="1"/>
+    </row>
+    <row r="108" ht="14.0" customFormat="1" s="18">
+      <c r="A108" s="8"/>
+      <c r="B108" s="8"/>
+      <c r="C108" s="8"/>
+      <c r="D108" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E108" s="12" t="s">
+        <v>62</v>
+      </c>
+      <c r="F108" s="19" t="s">
+        <v>100</v>
+      </c>
+      <c r="G108" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H108" s="8"/>
+      <c r="I108" s="10"/>
+      <c r="J108" s="1"/>
       <c r="K108" s="11"/>
       <c r="L108" s="11"/>
       <c r="M108" s="11"/>
@@ -5382,18 +6010,52 @@
       <c r="X108" s="11"/>
       <c r="Y108" s="11"/>
       <c r="Z108" s="11"/>
-    </row>
-    <row r="109" ht="14.0">
-      <c r="A109" s="11"/>
-      <c r="B109" s="11"/>
-      <c r="C109" s="11"/>
-      <c r="D109" s="11"/>
-      <c r="E109" s="11"/>
-      <c r="F109" s="11"/>
-      <c r="G109" s="11"/>
-      <c r="H109" s="11"/>
-      <c r="I109" s="11"/>
-      <c r="J109" s="11"/>
+      <c r="AA108" s="1"/>
+      <c r="AB108" s="1"/>
+      <c r="AC108" s="1"/>
+      <c r="AD108" s="1"/>
+      <c r="AE108" s="1"/>
+      <c r="AF108" s="1"/>
+      <c r="AG108" s="1"/>
+      <c r="AH108" s="1"/>
+      <c r="AI108" s="1"/>
+      <c r="AJ108" s="1"/>
+      <c r="AK108" s="1"/>
+      <c r="AL108" s="1"/>
+      <c r="AM108" s="1"/>
+      <c r="AN108" s="1"/>
+      <c r="AO108" s="1"/>
+      <c r="AP108" s="1"/>
+      <c r="AQ108" s="1"/>
+      <c r="AR108" s="1"/>
+      <c r="AS108" s="1"/>
+      <c r="AT108" s="1"/>
+      <c r="AU108" s="1"/>
+      <c r="AV108" s="1"/>
+      <c r="AW108" s="1"/>
+      <c r="AX108" s="1"/>
+      <c r="AY108" s="1"/>
+      <c r="AZ108" s="1"/>
+    </row>
+    <row r="109" ht="14.0" customFormat="1" s="18">
+      <c r="A109" s="8"/>
+      <c r="B109" s="8"/>
+      <c r="C109" s="8"/>
+      <c r="D109" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E109" s="12" t="s">
+        <v>65</v>
+      </c>
+      <c r="F109" s="8" t="s">
+        <v>102</v>
+      </c>
+      <c r="G109" s="9" t="s">
+        <v>101</v>
+      </c>
+      <c r="H109" s="8"/>
+      <c r="I109" s="10"/>
+      <c r="J109" s="1"/>
       <c r="K109" s="11"/>
       <c r="L109" s="11"/>
       <c r="M109" s="11"/>
@@ -5410,18 +6072,52 @@
       <c r="X109" s="11"/>
       <c r="Y109" s="11"/>
       <c r="Z109" s="11"/>
-    </row>
-    <row r="110" ht="14.0">
-      <c r="A110" s="11"/>
-      <c r="B110" s="11"/>
-      <c r="C110" s="11"/>
-      <c r="D110" s="11"/>
-      <c r="E110" s="11"/>
-      <c r="F110" s="11"/>
-      <c r="G110" s="11"/>
-      <c r="H110" s="11"/>
-      <c r="I110" s="11"/>
-      <c r="J110" s="11"/>
+      <c r="AA109" s="1"/>
+      <c r="AB109" s="1"/>
+      <c r="AC109" s="1"/>
+      <c r="AD109" s="1"/>
+      <c r="AE109" s="1"/>
+      <c r="AF109" s="1"/>
+      <c r="AG109" s="1"/>
+      <c r="AH109" s="1"/>
+      <c r="AI109" s="1"/>
+      <c r="AJ109" s="1"/>
+      <c r="AK109" s="1"/>
+      <c r="AL109" s="1"/>
+      <c r="AM109" s="1"/>
+      <c r="AN109" s="1"/>
+      <c r="AO109" s="1"/>
+      <c r="AP109" s="1"/>
+      <c r="AQ109" s="1"/>
+      <c r="AR109" s="1"/>
+      <c r="AS109" s="1"/>
+      <c r="AT109" s="1"/>
+      <c r="AU109" s="1"/>
+      <c r="AV109" s="1"/>
+      <c r="AW109" s="1"/>
+      <c r="AX109" s="1"/>
+      <c r="AY109" s="1"/>
+      <c r="AZ109" s="1"/>
+    </row>
+    <row r="110" ht="14.0" customFormat="1" s="18">
+      <c r="A110" s="8"/>
+      <c r="B110" s="8"/>
+      <c r="C110" s="8"/>
+      <c r="D110" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E110" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="F110" s="8" t="s">
+        <v>39</v>
+      </c>
+      <c r="G110" s="9" t="s">
+        <v>40</v>
+      </c>
+      <c r="H110" s="8"/>
+      <c r="I110" s="10"/>
+      <c r="J110" s="1"/>
       <c r="K110" s="11"/>
       <c r="L110" s="11"/>
       <c r="M110" s="11"/>
@@ -5438,18 +6134,52 @@
       <c r="X110" s="11"/>
       <c r="Y110" s="11"/>
       <c r="Z110" s="11"/>
-    </row>
-    <row r="111" ht="14.0">
-      <c r="A111" s="11"/>
-      <c r="B111" s="11"/>
-      <c r="C111" s="11"/>
-      <c r="D111" s="11"/>
-      <c r="E111" s="11"/>
-      <c r="F111" s="11"/>
-      <c r="G111" s="11"/>
-      <c r="H111" s="11"/>
-      <c r="I111" s="11"/>
-      <c r="J111" s="11"/>
+      <c r="AA110" s="1"/>
+      <c r="AB110" s="1"/>
+      <c r="AC110" s="1"/>
+      <c r="AD110" s="1"/>
+      <c r="AE110" s="1"/>
+      <c r="AF110" s="1"/>
+      <c r="AG110" s="1"/>
+      <c r="AH110" s="1"/>
+      <c r="AI110" s="1"/>
+      <c r="AJ110" s="1"/>
+      <c r="AK110" s="1"/>
+      <c r="AL110" s="1"/>
+      <c r="AM110" s="1"/>
+      <c r="AN110" s="1"/>
+      <c r="AO110" s="1"/>
+      <c r="AP110" s="1"/>
+      <c r="AQ110" s="1"/>
+      <c r="AR110" s="1"/>
+      <c r="AS110" s="1"/>
+      <c r="AT110" s="1"/>
+      <c r="AU110" s="1"/>
+      <c r="AV110" s="1"/>
+      <c r="AW110" s="1"/>
+      <c r="AX110" s="1"/>
+      <c r="AY110" s="1"/>
+      <c r="AZ110" s="1"/>
+    </row>
+    <row r="111" ht="14.0" customFormat="1" s="18">
+      <c r="A111" s="8"/>
+      <c r="B111" s="8"/>
+      <c r="C111" s="8"/>
+      <c r="D111" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E111" s="12" t="s">
+        <v>71</v>
+      </c>
+      <c r="F111" s="8" t="s">
+        <v>103</v>
+      </c>
+      <c r="G111" s="9" t="s">
+        <v>104</v>
+      </c>
+      <c r="H111" s="8"/>
+      <c r="I111" s="10"/>
+      <c r="J111" s="1"/>
       <c r="K111" s="11"/>
       <c r="L111" s="11"/>
       <c r="M111" s="11"/>
@@ -5466,18 +6196,52 @@
       <c r="X111" s="11"/>
       <c r="Y111" s="11"/>
       <c r="Z111" s="11"/>
-    </row>
-    <row r="112" ht="14.0">
-      <c r="A112" s="11"/>
-      <c r="B112" s="11"/>
-      <c r="C112" s="11"/>
-      <c r="D112" s="11"/>
-      <c r="E112" s="11"/>
-      <c r="F112" s="11"/>
-      <c r="G112" s="11"/>
-      <c r="H112" s="11"/>
-      <c r="I112" s="11"/>
-      <c r="J112" s="11"/>
+      <c r="AA111" s="1"/>
+      <c r="AB111" s="1"/>
+      <c r="AC111" s="1"/>
+      <c r="AD111" s="1"/>
+      <c r="AE111" s="1"/>
+      <c r="AF111" s="1"/>
+      <c r="AG111" s="1"/>
+      <c r="AH111" s="1"/>
+      <c r="AI111" s="1"/>
+      <c r="AJ111" s="1"/>
+      <c r="AK111" s="1"/>
+      <c r="AL111" s="1"/>
+      <c r="AM111" s="1"/>
+      <c r="AN111" s="1"/>
+      <c r="AO111" s="1"/>
+      <c r="AP111" s="1"/>
+      <c r="AQ111" s="1"/>
+      <c r="AR111" s="1"/>
+      <c r="AS111" s="1"/>
+      <c r="AT111" s="1"/>
+      <c r="AU111" s="1"/>
+      <c r="AV111" s="1"/>
+      <c r="AW111" s="1"/>
+      <c r="AX111" s="1"/>
+      <c r="AY111" s="1"/>
+      <c r="AZ111" s="1"/>
+    </row>
+    <row r="112" ht="14.0" customFormat="1" s="18">
+      <c r="A112" s="8"/>
+      <c r="B112" s="8"/>
+      <c r="C112" s="8"/>
+      <c r="D112" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E112" s="12" t="s">
+        <v>74</v>
+      </c>
+      <c r="F112" s="8" t="s">
+        <v>105</v>
+      </c>
+      <c r="G112" s="9" t="s">
+        <v>106</v>
+      </c>
+      <c r="H112" s="8"/>
+      <c r="I112" s="10"/>
+      <c r="J112" s="1"/>
       <c r="K112" s="11"/>
       <c r="L112" s="11"/>
       <c r="M112" s="11"/>
@@ -5494,18 +6258,52 @@
       <c r="X112" s="11"/>
       <c r="Y112" s="11"/>
       <c r="Z112" s="11"/>
-    </row>
-    <row r="113" ht="14.0">
-      <c r="A113" s="11"/>
-      <c r="B113" s="11"/>
-      <c r="C113" s="11"/>
-      <c r="D113" s="11"/>
-      <c r="E113" s="11"/>
-      <c r="F113" s="11"/>
-      <c r="G113" s="11"/>
-      <c r="H113" s="11"/>
-      <c r="I113" s="11"/>
-      <c r="J113" s="11"/>
+      <c r="AA112" s="1"/>
+      <c r="AB112" s="1"/>
+      <c r="AC112" s="1"/>
+      <c r="AD112" s="1"/>
+      <c r="AE112" s="1"/>
+      <c r="AF112" s="1"/>
+      <c r="AG112" s="1"/>
+      <c r="AH112" s="1"/>
+      <c r="AI112" s="1"/>
+      <c r="AJ112" s="1"/>
+      <c r="AK112" s="1"/>
+      <c r="AL112" s="1"/>
+      <c r="AM112" s="1"/>
+      <c r="AN112" s="1"/>
+      <c r="AO112" s="1"/>
+      <c r="AP112" s="1"/>
+      <c r="AQ112" s="1"/>
+      <c r="AR112" s="1"/>
+      <c r="AS112" s="1"/>
+      <c r="AT112" s="1"/>
+      <c r="AU112" s="1"/>
+      <c r="AV112" s="1"/>
+      <c r="AW112" s="1"/>
+      <c r="AX112" s="1"/>
+      <c r="AY112" s="1"/>
+      <c r="AZ112" s="1"/>
+    </row>
+    <row r="113" ht="14.0" customFormat="1" s="18">
+      <c r="A113" s="8"/>
+      <c r="B113" s="8"/>
+      <c r="C113" s="8"/>
+      <c r="D113" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E113" s="12" t="s">
+        <v>77</v>
+      </c>
+      <c r="F113" s="8" t="s">
+        <v>107</v>
+      </c>
+      <c r="G113" s="9" t="s">
+        <v>108</v>
+      </c>
+      <c r="H113" s="8"/>
+      <c r="I113" s="10"/>
+      <c r="J113" s="1"/>
       <c r="K113" s="11"/>
       <c r="L113" s="11"/>
       <c r="M113" s="11"/>
@@ -5522,18 +6320,52 @@
       <c r="X113" s="11"/>
       <c r="Y113" s="11"/>
       <c r="Z113" s="11"/>
-    </row>
-    <row r="114" ht="14.0">
-      <c r="A114" s="11"/>
-      <c r="B114" s="11"/>
-      <c r="C114" s="11"/>
-      <c r="D114" s="11"/>
-      <c r="E114" s="11"/>
-      <c r="F114" s="11"/>
-      <c r="G114" s="11"/>
-      <c r="H114" s="11"/>
-      <c r="I114" s="11"/>
-      <c r="J114" s="11"/>
+      <c r="AA113" s="1"/>
+      <c r="AB113" s="1"/>
+      <c r="AC113" s="1"/>
+      <c r="AD113" s="1"/>
+      <c r="AE113" s="1"/>
+      <c r="AF113" s="1"/>
+      <c r="AG113" s="1"/>
+      <c r="AH113" s="1"/>
+      <c r="AI113" s="1"/>
+      <c r="AJ113" s="1"/>
+      <c r="AK113" s="1"/>
+      <c r="AL113" s="1"/>
+      <c r="AM113" s="1"/>
+      <c r="AN113" s="1"/>
+      <c r="AO113" s="1"/>
+      <c r="AP113" s="1"/>
+      <c r="AQ113" s="1"/>
+      <c r="AR113" s="1"/>
+      <c r="AS113" s="1"/>
+      <c r="AT113" s="1"/>
+      <c r="AU113" s="1"/>
+      <c r="AV113" s="1"/>
+      <c r="AW113" s="1"/>
+      <c r="AX113" s="1"/>
+      <c r="AY113" s="1"/>
+      <c r="AZ113" s="1"/>
+    </row>
+    <row r="114" ht="14.0" customFormat="1" s="18">
+      <c r="A114" s="8"/>
+      <c r="B114" s="8"/>
+      <c r="C114" s="8"/>
+      <c r="D114" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E114" s="12" t="s">
+        <v>80</v>
+      </c>
+      <c r="F114" s="8" t="s">
+        <v>109</v>
+      </c>
+      <c r="G114" s="9" t="s">
+        <v>110</v>
+      </c>
+      <c r="H114" s="8"/>
+      <c r="I114" s="10"/>
+      <c r="J114" s="1"/>
       <c r="K114" s="11"/>
       <c r="L114" s="11"/>
       <c r="M114" s="11"/>
@@ -5550,18 +6382,52 @@
       <c r="X114" s="11"/>
       <c r="Y114" s="11"/>
       <c r="Z114" s="11"/>
-    </row>
-    <row r="115" ht="14.0">
-      <c r="A115" s="11"/>
-      <c r="B115" s="11"/>
-      <c r="C115" s="11"/>
-      <c r="D115" s="11"/>
-      <c r="E115" s="11"/>
-      <c r="F115" s="11"/>
-      <c r="G115" s="11"/>
-      <c r="H115" s="11"/>
-      <c r="I115" s="11"/>
-      <c r="J115" s="11"/>
+      <c r="AA114" s="1"/>
+      <c r="AB114" s="1"/>
+      <c r="AC114" s="1"/>
+      <c r="AD114" s="1"/>
+      <c r="AE114" s="1"/>
+      <c r="AF114" s="1"/>
+      <c r="AG114" s="1"/>
+      <c r="AH114" s="1"/>
+      <c r="AI114" s="1"/>
+      <c r="AJ114" s="1"/>
+      <c r="AK114" s="1"/>
+      <c r="AL114" s="1"/>
+      <c r="AM114" s="1"/>
+      <c r="AN114" s="1"/>
+      <c r="AO114" s="1"/>
+      <c r="AP114" s="1"/>
+      <c r="AQ114" s="1"/>
+      <c r="AR114" s="1"/>
+      <c r="AS114" s="1"/>
+      <c r="AT114" s="1"/>
+      <c r="AU114" s="1"/>
+      <c r="AV114" s="1"/>
+      <c r="AW114" s="1"/>
+      <c r="AX114" s="1"/>
+      <c r="AY114" s="1"/>
+      <c r="AZ114" s="1"/>
+    </row>
+    <row r="115" ht="14.0" customFormat="1" s="18">
+      <c r="A115" s="8"/>
+      <c r="B115" s="8"/>
+      <c r="C115" s="8"/>
+      <c r="D115" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E115" s="12" t="s">
+        <v>83</v>
+      </c>
+      <c r="F115" s="8" t="s">
+        <v>111</v>
+      </c>
+      <c r="G115" s="9" t="s">
+        <v>112</v>
+      </c>
+      <c r="H115" s="8"/>
+      <c r="I115" s="10"/>
+      <c r="J115" s="1"/>
       <c r="K115" s="11"/>
       <c r="L115" s="11"/>
       <c r="M115" s="11"/>
@@ -5578,18 +6444,52 @@
       <c r="X115" s="11"/>
       <c r="Y115" s="11"/>
       <c r="Z115" s="11"/>
-    </row>
-    <row r="116" ht="14.0">
-      <c r="A116" s="11"/>
-      <c r="B116" s="11"/>
-      <c r="C116" s="11"/>
-      <c r="D116" s="11"/>
-      <c r="E116" s="11"/>
-      <c r="F116" s="11"/>
-      <c r="G116" s="11"/>
-      <c r="H116" s="11"/>
-      <c r="I116" s="11"/>
-      <c r="J116" s="11"/>
+      <c r="AA115" s="1"/>
+      <c r="AB115" s="1"/>
+      <c r="AC115" s="1"/>
+      <c r="AD115" s="1"/>
+      <c r="AE115" s="1"/>
+      <c r="AF115" s="1"/>
+      <c r="AG115" s="1"/>
+      <c r="AH115" s="1"/>
+      <c r="AI115" s="1"/>
+      <c r="AJ115" s="1"/>
+      <c r="AK115" s="1"/>
+      <c r="AL115" s="1"/>
+      <c r="AM115" s="1"/>
+      <c r="AN115" s="1"/>
+      <c r="AO115" s="1"/>
+      <c r="AP115" s="1"/>
+      <c r="AQ115" s="1"/>
+      <c r="AR115" s="1"/>
+      <c r="AS115" s="1"/>
+      <c r="AT115" s="1"/>
+      <c r="AU115" s="1"/>
+      <c r="AV115" s="1"/>
+      <c r="AW115" s="1"/>
+      <c r="AX115" s="1"/>
+      <c r="AY115" s="1"/>
+      <c r="AZ115" s="1"/>
+    </row>
+    <row r="116" ht="14.0" customFormat="1" s="18">
+      <c r="A116" s="8"/>
+      <c r="B116" s="8"/>
+      <c r="C116" s="8"/>
+      <c r="D116" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E116" s="12" t="s">
+        <v>86</v>
+      </c>
+      <c r="F116" s="8" t="s">
+        <v>152</v>
+      </c>
+      <c r="G116" s="9" t="s">
+        <v>114</v>
+      </c>
+      <c r="H116" s="8"/>
+      <c r="I116" s="10"/>
+      <c r="J116" s="1"/>
       <c r="K116" s="11"/>
       <c r="L116" s="11"/>
       <c r="M116" s="11"/>
@@ -5606,18 +6506,52 @@
       <c r="X116" s="11"/>
       <c r="Y116" s="11"/>
       <c r="Z116" s="11"/>
-    </row>
-    <row r="117" ht="14.0">
-      <c r="A117" s="11"/>
-      <c r="B117" s="11"/>
-      <c r="C117" s="11"/>
-      <c r="D117" s="11"/>
-      <c r="E117" s="11"/>
-      <c r="F117" s="11"/>
-      <c r="G117" s="11"/>
-      <c r="H117" s="11"/>
-      <c r="I117" s="11"/>
-      <c r="J117" s="11"/>
+      <c r="AA116" s="1"/>
+      <c r="AB116" s="1"/>
+      <c r="AC116" s="1"/>
+      <c r="AD116" s="1"/>
+      <c r="AE116" s="1"/>
+      <c r="AF116" s="1"/>
+      <c r="AG116" s="1"/>
+      <c r="AH116" s="1"/>
+      <c r="AI116" s="1"/>
+      <c r="AJ116" s="1"/>
+      <c r="AK116" s="1"/>
+      <c r="AL116" s="1"/>
+      <c r="AM116" s="1"/>
+      <c r="AN116" s="1"/>
+      <c r="AO116" s="1"/>
+      <c r="AP116" s="1"/>
+      <c r="AQ116" s="1"/>
+      <c r="AR116" s="1"/>
+      <c r="AS116" s="1"/>
+      <c r="AT116" s="1"/>
+      <c r="AU116" s="1"/>
+      <c r="AV116" s="1"/>
+      <c r="AW116" s="1"/>
+      <c r="AX116" s="1"/>
+      <c r="AY116" s="1"/>
+      <c r="AZ116" s="1"/>
+    </row>
+    <row r="117" ht="14.0" customFormat="1" s="18">
+      <c r="A117" s="8"/>
+      <c r="B117" s="8"/>
+      <c r="C117" s="8"/>
+      <c r="D117" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E117" s="12" t="s">
+        <v>115</v>
+      </c>
+      <c r="F117" s="8" t="s">
+        <v>153</v>
+      </c>
+      <c r="G117" s="9" t="s">
+        <v>117</v>
+      </c>
+      <c r="H117" s="8"/>
+      <c r="I117" s="10"/>
+      <c r="J117" s="1"/>
       <c r="K117" s="11"/>
       <c r="L117" s="11"/>
       <c r="M117" s="11"/>
@@ -5634,18 +6568,52 @@
       <c r="X117" s="11"/>
       <c r="Y117" s="11"/>
       <c r="Z117" s="11"/>
-    </row>
-    <row r="118" ht="14.0">
-      <c r="A118" s="11"/>
-      <c r="B118" s="11"/>
-      <c r="C118" s="11"/>
-      <c r="D118" s="11"/>
-      <c r="E118" s="11"/>
-      <c r="F118" s="11"/>
-      <c r="G118" s="11"/>
-      <c r="H118" s="11"/>
-      <c r="I118" s="11"/>
-      <c r="J118" s="11"/>
+      <c r="AA117" s="1"/>
+      <c r="AB117" s="1"/>
+      <c r="AC117" s="1"/>
+      <c r="AD117" s="1"/>
+      <c r="AE117" s="1"/>
+      <c r="AF117" s="1"/>
+      <c r="AG117" s="1"/>
+      <c r="AH117" s="1"/>
+      <c r="AI117" s="1"/>
+      <c r="AJ117" s="1"/>
+      <c r="AK117" s="1"/>
+      <c r="AL117" s="1"/>
+      <c r="AM117" s="1"/>
+      <c r="AN117" s="1"/>
+      <c r="AO117" s="1"/>
+      <c r="AP117" s="1"/>
+      <c r="AQ117" s="1"/>
+      <c r="AR117" s="1"/>
+      <c r="AS117" s="1"/>
+      <c r="AT117" s="1"/>
+      <c r="AU117" s="1"/>
+      <c r="AV117" s="1"/>
+      <c r="AW117" s="1"/>
+      <c r="AX117" s="1"/>
+      <c r="AY117" s="1"/>
+      <c r="AZ117" s="1"/>
+    </row>
+    <row r="118" ht="14.0" customFormat="1" s="18">
+      <c r="A118" s="8"/>
+      <c r="B118" s="8"/>
+      <c r="C118" s="8"/>
+      <c r="D118" s="12" t="s">
+        <v>13</v>
+      </c>
+      <c r="E118" s="12" t="s">
+        <v>118</v>
+      </c>
+      <c r="F118" s="8" t="s">
+        <v>119</v>
+      </c>
+      <c r="G118" s="9" t="s">
+        <v>120</v>
+      </c>
+      <c r="H118" s="8"/>
+      <c r="I118" s="10"/>
+      <c r="J118" s="1"/>
       <c r="K118" s="11"/>
       <c r="L118" s="11"/>
       <c r="M118" s="11"/>
@@ -5662,6 +6630,32 @@
       <c r="X118" s="11"/>
       <c r="Y118" s="11"/>
       <c r="Z118" s="11"/>
+      <c r="AA118" s="1"/>
+      <c r="AB118" s="1"/>
+      <c r="AC118" s="1"/>
+      <c r="AD118" s="1"/>
+      <c r="AE118" s="1"/>
+      <c r="AF118" s="1"/>
+      <c r="AG118" s="1"/>
+      <c r="AH118" s="1"/>
+      <c r="AI118" s="1"/>
+      <c r="AJ118" s="1"/>
+      <c r="AK118" s="1"/>
+      <c r="AL118" s="1"/>
+      <c r="AM118" s="1"/>
+      <c r="AN118" s="1"/>
+      <c r="AO118" s="1"/>
+      <c r="AP118" s="1"/>
+      <c r="AQ118" s="1"/>
+      <c r="AR118" s="1"/>
+      <c r="AS118" s="1"/>
+      <c r="AT118" s="1"/>
+      <c r="AU118" s="1"/>
+      <c r="AV118" s="1"/>
+      <c r="AW118" s="1"/>
+      <c r="AX118" s="1"/>
+      <c r="AY118" s="1"/>
+      <c r="AZ118" s="1"/>
     </row>
     <row r="119" ht="14.0">
       <c r="A119" s="11"/>
@@ -10732,90 +11726,90 @@
       <c r="Z299" s="11"/>
     </row>
     <row r="300" ht="14.0">
-      <c r="A300" s="19">
+      <c r="A300" s="20">
         <f>COUNTA(A2:A299)</f>
-        <v>3.0</v>
-      </c>
-      <c r="B300" s="19"/>
-      <c r="C300" s="19"/>
-      <c r="D300" s="19"/>
-      <c r="E300" s="19"/>
-      <c r="F300" s="19"/>
-      <c r="G300" s="19"/>
-      <c r="H300" s="19">
+        <v>4.0</v>
+      </c>
+      <c r="B300" s="20"/>
+      <c r="C300" s="20"/>
+      <c r="D300" s="20"/>
+      <c r="E300" s="20"/>
+      <c r="F300" s="20"/>
+      <c r="G300" s="20"/>
+      <c r="H300" s="20">
         <f>COUNTA(H313:H593)</f>
         <v>0.0</v>
       </c>
-      <c r="I300" s="19"/>
-      <c r="J300" s="19"/>
-      <c r="K300" s="19"/>
-      <c r="L300" s="19"/>
-      <c r="M300" s="19"/>
-      <c r="N300" s="19"/>
-      <c r="O300" s="19"/>
-      <c r="P300" s="19"/>
-      <c r="Q300" s="19"/>
-      <c r="R300" s="19"/>
-      <c r="S300" s="19"/>
-      <c r="T300" s="19"/>
-      <c r="U300" s="19"/>
-      <c r="V300" s="19"/>
-      <c r="W300" s="19"/>
-      <c r="X300" s="19"/>
-      <c r="Y300" s="19"/>
-      <c r="Z300" s="19"/>
-      <c r="AA300" s="20"/>
-      <c r="AB300" s="20"/>
-      <c r="AC300" s="20"/>
-      <c r="AD300" s="20"/>
-      <c r="AE300" s="20"/>
-      <c r="AF300" s="20"/>
-      <c r="AG300" s="20"/>
-      <c r="AH300" s="20"/>
-      <c r="AI300" s="20"/>
-      <c r="AJ300" s="20"/>
-      <c r="AK300" s="20"/>
-      <c r="AL300" s="20"/>
-      <c r="AM300" s="20"/>
-      <c r="AN300" s="20"/>
-      <c r="AO300" s="20"/>
-      <c r="AP300" s="20"/>
-      <c r="AQ300" s="20"/>
-      <c r="AR300" s="20"/>
-      <c r="AS300" s="20"/>
-      <c r="AT300" s="20"/>
-      <c r="AU300" s="20"/>
-      <c r="AV300" s="20"/>
-      <c r="AW300" s="20"/>
-      <c r="AX300" s="20"/>
-      <c r="AY300" s="20"/>
-      <c r="AZ300" s="20"/>
-      <c r="IW300" s="21"/>
-      <c r="IX300" s="21"/>
-      <c r="IY300" s="21"/>
-      <c r="IZ300" s="21"/>
-      <c r="JA300" s="21"/>
-      <c r="JB300" s="21"/>
-      <c r="JC300" s="21"/>
-      <c r="JD300" s="21"/>
-      <c r="JE300" s="21"/>
-      <c r="JF300" s="21"/>
-      <c r="JG300" s="21"/>
-      <c r="JH300" s="21"/>
-      <c r="JI300" s="21"/>
-      <c r="JJ300" s="21"/>
-      <c r="JK300" s="21"/>
-      <c r="JL300" s="21"/>
-      <c r="JM300" s="21"/>
-      <c r="JN300" s="21"/>
-      <c r="JO300" s="21"/>
-      <c r="JP300" s="21"/>
-      <c r="JQ300" s="21"/>
-      <c r="JR300" s="21"/>
-      <c r="JS300" s="21"/>
-      <c r="JT300" s="21"/>
-      <c r="JU300" s="21"/>
-      <c r="JV300" s="21"/>
+      <c r="I300" s="20"/>
+      <c r="J300" s="20"/>
+      <c r="K300" s="20"/>
+      <c r="L300" s="20"/>
+      <c r="M300" s="20"/>
+      <c r="N300" s="20"/>
+      <c r="O300" s="20"/>
+      <c r="P300" s="20"/>
+      <c r="Q300" s="20"/>
+      <c r="R300" s="20"/>
+      <c r="S300" s="20"/>
+      <c r="T300" s="20"/>
+      <c r="U300" s="20"/>
+      <c r="V300" s="20"/>
+      <c r="W300" s="20"/>
+      <c r="X300" s="20"/>
+      <c r="Y300" s="20"/>
+      <c r="Z300" s="20"/>
+      <c r="AA300" s="21"/>
+      <c r="AB300" s="21"/>
+      <c r="AC300" s="21"/>
+      <c r="AD300" s="21"/>
+      <c r="AE300" s="21"/>
+      <c r="AF300" s="21"/>
+      <c r="AG300" s="21"/>
+      <c r="AH300" s="21"/>
+      <c r="AI300" s="21"/>
+      <c r="AJ300" s="21"/>
+      <c r="AK300" s="21"/>
+      <c r="AL300" s="21"/>
+      <c r="AM300" s="21"/>
+      <c r="AN300" s="21"/>
+      <c r="AO300" s="21"/>
+      <c r="AP300" s="21"/>
+      <c r="AQ300" s="21"/>
+      <c r="AR300" s="21"/>
+      <c r="AS300" s="21"/>
+      <c r="AT300" s="21"/>
+      <c r="AU300" s="21"/>
+      <c r="AV300" s="21"/>
+      <c r="AW300" s="21"/>
+      <c r="AX300" s="21"/>
+      <c r="AY300" s="21"/>
+      <c r="AZ300" s="21"/>
+      <c r="IW300" s="22"/>
+      <c r="IX300" s="22"/>
+      <c r="IY300" s="22"/>
+      <c r="IZ300" s="22"/>
+      <c r="JA300" s="22"/>
+      <c r="JB300" s="22"/>
+      <c r="JC300" s="22"/>
+      <c r="JD300" s="22"/>
+      <c r="JE300" s="22"/>
+      <c r="JF300" s="22"/>
+      <c r="JG300" s="22"/>
+      <c r="JH300" s="22"/>
+      <c r="JI300" s="22"/>
+      <c r="JJ300" s="22"/>
+      <c r="JK300" s="22"/>
+      <c r="JL300" s="22"/>
+      <c r="JM300" s="22"/>
+      <c r="JN300" s="22"/>
+      <c r="JO300" s="22"/>
+      <c r="JP300" s="22"/>
+      <c r="JQ300" s="22"/>
+      <c r="JR300" s="22"/>
+      <c r="JS300" s="22"/>
+      <c r="JT300" s="22"/>
+      <c r="JU300" s="22"/>
+      <c r="JV300" s="22"/>
     </row>
     <row r="301" ht="14.0">
       <c r="A301" s="11"/>
@@ -25560,6 +26554,7 @@
   <hyperlinks>
     <hyperlink ref="F45" r:id="rId1"/>
     <hyperlink ref="F80" r:id="rId2"/>
+    <hyperlink ref="F108" r:id="rId3"/>
   </hyperlinks>
   <extLst/>
 </worksheet>

</xml_diff>